<commit_message>
add 047 ~ 049
</commit_message>
<xml_diff>
--- a/graphdb_inputs/meta-model.xlsx
+++ b/graphdb_inputs/meta-model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\EA_MetaModel\graphdb_inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431C87EB-E84B-4537-B396-69680F2DD79C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95EEE15-BA8C-438F-8F53-D8A0C9BD157B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11670" yWindow="0" windowWidth="17115" windowHeight="15585" xr2:uid="{8170F98D-87F3-4BBF-AF33-E74360046B09}"/>
+    <workbookView xWindow="3780" yWindow="3015" windowWidth="19740" windowHeight="11295" xr2:uid="{8170F98D-87F3-4BBF-AF33-E74360046B09}"/>
   </bookViews>
   <sheets>
     <sheet name="meta-model" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="132">
   <si>
     <t>source</t>
   </si>
@@ -411,6 +411,27 @@
   </si>
   <si>
     <t>Application_Provider_Role</t>
+  </si>
+  <si>
+    <t>Static_Application_Provider_Architecture</t>
+  </si>
+  <si>
+    <t>:APA-STATIC-RELATION</t>
+  </si>
+  <si>
+    <t>:Application_Relationship</t>
+  </si>
+  <si>
+    <t>Logical Software Architecture</t>
+  </si>
+  <si>
+    <t>SCA RELATION</t>
+  </si>
+  <si>
+    <t>Application_Function_Implementation</t>
+  </si>
+  <si>
+    <t>Application_Function</t>
   </si>
 </sst>
 </file>
@@ -780,8 +801,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AB3976EA-2B8D-46CC-B8F3-0DB3881E99F9}" name="Table1" displayName="Table1" ref="A1:E177" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6" totalsRowBorderDxfId="5">
-  <autoFilter ref="A1:E177" xr:uid="{AB3976EA-2B8D-46CC-B8F3-0DB3881E99F9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AB3976EA-2B8D-46CC-B8F3-0DB3881E99F9}" name="Table1" displayName="Table1" ref="A1:E189" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6" totalsRowBorderDxfId="5">
+  <autoFilter ref="A1:E189" xr:uid="{AB3976EA-2B8D-46CC-B8F3-0DB3881E99F9}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{768FEF15-CE91-4610-9962-A2388F3D8C76}" name="source" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{6BA5C30C-3AC2-4B96-8F4B-FB5D1FBD553E}" name="source_label" dataDxfId="3"/>
@@ -1110,13 +1131,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3C6A4DC-C1A5-4591-B4CB-A04A3C9852DB}">
-  <dimension ref="A1:E177"/>
+  <dimension ref="A1:E189"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.7109375" customWidth="1"/>
     <col min="2" max="2" width="23.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.5703125" customWidth="1"/>
+    <col min="4" max="4" width="37.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4126,6 +4147,210 @@
         <v>124</v>
       </c>
       <c r="E177" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B178" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C178" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D178" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E178" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B179" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C179" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D179" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E179" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B180" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C180" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D180" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E180" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A181" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B181" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C181" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D181" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E181" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A182" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B182" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C182" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D182" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="E182" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A183" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B183" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C183" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D183" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E183" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A184" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B184" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C184" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D184" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="E184" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A185" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B185" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C185" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D185" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E185" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A186" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B186" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C186" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D186" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="E186" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A187" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B187" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C187" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D187" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E187" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A188" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B188" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C188" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="D188" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="E188" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A189" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B189" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C189" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D189" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="E189" s="9" t="s">
         <v>96</v>
       </c>
     </row>

</xml_diff>